<commit_message>
Correct LaborHrsPerBedCarrots, OwnWageRate and TempWageRate in model.xlsx
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EUWMPsy2iAZCcY5yjMvY5G
</commit_message>
<xml_diff>
--- a/capabilities/marginal-analysis/model.xlsx
+++ b/capabilities/marginal-analysis/model.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mysp-cloud.kp.org/personal/ryan_m_moore_kp_org/Documents/Shidler/BUS 620 Econ Foundations/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{42EFEC8F-C093-48B7-945B-F1A08FF85ADD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AD3EF3D2-DFF6-4E04-94CE-5D6D7E9A6441}"/>
+  <xr:revisionPtr revIDLastSave="9" documentId="13_ncr:1_{42EFEC8F-C093-48B7-945B-F1A08FF85ADD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5EB91849-C687-4229-9A96-0F12D5E57DBB}"/>
   <bookViews>
     <workbookView xWindow="22932" yWindow="1272" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -399,8 +399,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="\$#,##0"/>
+    <numFmt numFmtId="166" formatCode="\$#,##0.00"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -437,7 +438,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -450,6 +451,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="166" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -824,7 +826,8 @@
         <v>2094</v>
       </c>
       <c r="D6" s="3">
-        <v>0.83299999999999996</v>
+        <f>2.5/3</f>
+        <v>0.83333333333333337</v>
       </c>
       <c r="E6" s="3">
         <v>440</v>
@@ -895,7 +898,8 @@
         <v>16</v>
       </c>
       <c r="B14" s="3">
-        <v>34.72</v>
+        <f>25000/720</f>
+        <v>34.722222222222221</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
@@ -919,7 +923,8 @@
         <v>19</v>
       </c>
       <c r="B17" s="3">
-        <v>17.36</v>
+        <f>25000/1440</f>
+        <v>17.361111111111111</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
@@ -1009,7 +1014,7 @@
       </c>
       <c r="B10" s="3">
         <f>BedsCarrots*LaborHrsPerBedCarrots*SeasonWeeks*(1+DimReturnsCarrots)^BedsCarrots</f>
-        <v>982.77659622856766</v>
+        <v>983.16986417423732</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
@@ -1027,7 +1032,7 @@
       </c>
       <c r="B12" s="6">
         <f>LaborHoursTomatoes+LaborHoursCarrots+LaborHoursMesclun</f>
-        <v>5276.8228463282185</v>
+        <v>5277.2161142738878</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
@@ -1050,7 +1055,7 @@
       </c>
       <c r="B16" s="3">
         <f>MAX(TotalLaborHours-OwnLaborHours,0)</f>
-        <v>4556.8228463282185</v>
+        <v>4557.2161142738878</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
@@ -1068,7 +1073,7 @@
       </c>
       <c r="B18" s="7">
         <f>OwnLaborHoursUsed*OwnWageRate+TempLaborHoursUsed*TempWageRate</f>
-        <v>104104.84461225786</v>
+        <v>104118.335317255</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
@@ -1100,16 +1105,16 @@
       </c>
       <c r="B23" s="7">
         <f>FixedCosts+FertilizerCost+LaborCost</f>
-        <v>168104.84461225785</v>
+        <v>168118.335317255</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="B24" s="7">
+      <c r="B24" s="10">
         <f>Revenue-TotalCost</f>
-        <v>42775.155387742154</v>
+        <v>42761.664682745002</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
@@ -1308,7 +1313,7 @@
       </c>
       <c r="B22" s="3">
         <f>TotalLaborHours</f>
-        <v>5276.8228463282185</v>
+        <v>5277.2161142738878</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.3">
@@ -1326,7 +1331,7 @@
       </c>
       <c r="B24" s="5">
         <f>TotalCost</f>
-        <v>168104.84461225785</v>
+        <v>168118.335317255</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.3">
@@ -1335,7 +1340,7 @@
       </c>
       <c r="B25" s="7">
         <f>Profit</f>
-        <v>42775.155387742154</v>
+        <v>42761.664682745002</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Remove empty Solver model from Output sheet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EUWMPsy2iAZCcY5yjMvY5G
</commit_message>
<xml_diff>
--- a/capabilities/marginal-analysis/model.xlsx
+++ b/capabilities/marginal-analysis/model.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mysp-cloud.kp.org/personal/ryan_m_moore_kp_org/Documents/Shidler/BUS 620 Econ Foundations/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="9" documentId="13_ncr:1_{42EFEC8F-C093-48B7-945B-F1A08FF85ADD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5EB91849-C687-4229-9A96-0F12D5E57DBB}"/>
+  <xr:revisionPtr revIDLastSave="32" documentId="13_ncr:1_{42EFEC8F-C093-48B7-945B-F1A08FF85ADD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4B0D96A2-9374-48DC-95F6-3C644B37B340}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="1272" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22932" yWindow="1272" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Inputs" sheetId="1" r:id="rId1"/>
@@ -50,92 +50,52 @@
     <definedName name="SeasonWeeks">Inputs!$B$12</definedName>
     <definedName name="solver_adj" localSheetId="1" hidden="1">Calc!$B$4:$B$6</definedName>
     <definedName name="solver_cvg" localSheetId="1" hidden="1">0.0001</definedName>
-    <definedName name="solver_cvg" localSheetId="2" hidden="1">0.0001</definedName>
     <definedName name="solver_drv" localSheetId="1" hidden="1">1</definedName>
-    <definedName name="solver_drv" localSheetId="2" hidden="1">2</definedName>
     <definedName name="solver_eng" localSheetId="1" hidden="1">1</definedName>
-    <definedName name="solver_eng" localSheetId="2" hidden="1">1</definedName>
     <definedName name="solver_est" localSheetId="1" hidden="1">1</definedName>
-    <definedName name="solver_est" localSheetId="2" hidden="1">1</definedName>
     <definedName name="solver_itr" localSheetId="1" hidden="1">2147483647</definedName>
-    <definedName name="solver_itr" localSheetId="2" hidden="1">2147483647</definedName>
     <definedName name="solver_lhs1" localSheetId="1" hidden="1">Calc!$B$4:$B$6</definedName>
-    <definedName name="solver_lhs1" localSheetId="2" hidden="1">Output!$B$6</definedName>
     <definedName name="solver_lhs2" localSheetId="1" hidden="1">Calc!$B$4:$B$6</definedName>
-    <definedName name="solver_lhs2" localSheetId="2" hidden="1">Output!$B$6</definedName>
     <definedName name="solver_lhs3" localSheetId="1" hidden="1">Calc!$B$5</definedName>
-    <definedName name="solver_lhs3" localSheetId="2" hidden="1">Output!$B$6</definedName>
     <definedName name="solver_lhs4" localSheetId="1" hidden="1">Calc!$B$6</definedName>
-    <definedName name="solver_lhs4" localSheetId="2" hidden="1">Output!$B$6</definedName>
     <definedName name="solver_lhs5" localSheetId="1" hidden="1">Calc!$B$4</definedName>
-    <definedName name="solver_lhs5" localSheetId="2" hidden="1">Output!$B$6</definedName>
     <definedName name="solver_lhs6" localSheetId="1" hidden="1">Calc!$B$27</definedName>
     <definedName name="solver_lhs7" localSheetId="1" hidden="1">Calc!$B$12</definedName>
     <definedName name="solver_mip" localSheetId="1" hidden="1">2147483647</definedName>
-    <definedName name="solver_mip" localSheetId="2" hidden="1">2147483647</definedName>
     <definedName name="solver_mni" localSheetId="1" hidden="1">30</definedName>
-    <definedName name="solver_mni" localSheetId="2" hidden="1">30</definedName>
     <definedName name="solver_mrt" localSheetId="1" hidden="1">0.075</definedName>
-    <definedName name="solver_mrt" localSheetId="2" hidden="1">0.075</definedName>
     <definedName name="solver_msl" localSheetId="1" hidden="1">2</definedName>
-    <definedName name="solver_msl" localSheetId="2" hidden="1">2</definedName>
     <definedName name="solver_neg" localSheetId="1" hidden="1">1</definedName>
-    <definedName name="solver_neg" localSheetId="2" hidden="1">1</definedName>
     <definedName name="solver_nod" localSheetId="1" hidden="1">2147483647</definedName>
-    <definedName name="solver_nod" localSheetId="2" hidden="1">2147483647</definedName>
     <definedName name="solver_num" localSheetId="1" hidden="1">7</definedName>
-    <definedName name="solver_num" localSheetId="2" hidden="1">0</definedName>
     <definedName name="solver_nwt" localSheetId="1" hidden="1">1</definedName>
-    <definedName name="solver_nwt" localSheetId="2" hidden="1">1</definedName>
     <definedName name="solver_opt" localSheetId="1" hidden="1">Calc!$B$24</definedName>
     <definedName name="solver_pre" localSheetId="1" hidden="1">0.000001</definedName>
-    <definedName name="solver_pre" localSheetId="2" hidden="1">0.000001</definedName>
     <definedName name="solver_rbv" localSheetId="1" hidden="1">1</definedName>
-    <definedName name="solver_rbv" localSheetId="2" hidden="1">2</definedName>
     <definedName name="solver_rel1" localSheetId="1" hidden="1">4</definedName>
-    <definedName name="solver_rel1" localSheetId="2" hidden="1">1</definedName>
     <definedName name="solver_rel2" localSheetId="1" hidden="1">3</definedName>
-    <definedName name="solver_rel2" localSheetId="2" hidden="1">1</definedName>
     <definedName name="solver_rel3" localSheetId="1" hidden="1">1</definedName>
-    <definedName name="solver_rel3" localSheetId="2" hidden="1">1</definedName>
     <definedName name="solver_rel4" localSheetId="1" hidden="1">1</definedName>
-    <definedName name="solver_rel4" localSheetId="2" hidden="1">1</definedName>
     <definedName name="solver_rel5" localSheetId="1" hidden="1">1</definedName>
-    <definedName name="solver_rel5" localSheetId="2" hidden="1">1</definedName>
     <definedName name="solver_rel6" localSheetId="1" hidden="1">1</definedName>
     <definedName name="solver_rel7" localSheetId="1" hidden="1">1</definedName>
     <definedName name="solver_rhs1" localSheetId="1" hidden="1">"integer"</definedName>
-    <definedName name="solver_rhs1" localSheetId="2" hidden="1">30</definedName>
     <definedName name="solver_rhs2" localSheetId="1" hidden="1">0</definedName>
-    <definedName name="solver_rhs2" localSheetId="2" hidden="1">30</definedName>
     <definedName name="solver_rhs3" localSheetId="1" hidden="1">20</definedName>
-    <definedName name="solver_rhs3" localSheetId="2" hidden="1">30</definedName>
     <definedName name="solver_rhs4" localSheetId="1" hidden="1">30</definedName>
-    <definedName name="solver_rhs4" localSheetId="2" hidden="1">30</definedName>
     <definedName name="solver_rhs5" localSheetId="1" hidden="1">20</definedName>
-    <definedName name="solver_rhs5" localSheetId="2" hidden="1">30</definedName>
     <definedName name="solver_rhs6" localSheetId="1" hidden="1">64</definedName>
     <definedName name="solver_rhs7" localSheetId="1" hidden="1">TotalLaborCapacity</definedName>
     <definedName name="solver_rlx" localSheetId="1" hidden="1">2</definedName>
-    <definedName name="solver_rlx" localSheetId="2" hidden="1">2</definedName>
     <definedName name="solver_rsd" localSheetId="1" hidden="1">0</definedName>
-    <definedName name="solver_rsd" localSheetId="2" hidden="1">0</definedName>
     <definedName name="solver_scl" localSheetId="1" hidden="1">1</definedName>
-    <definedName name="solver_scl" localSheetId="2" hidden="1">2</definedName>
     <definedName name="solver_sho" localSheetId="1" hidden="1">2</definedName>
-    <definedName name="solver_sho" localSheetId="2" hidden="1">2</definedName>
     <definedName name="solver_ssz" localSheetId="1" hidden="1">100</definedName>
-    <definedName name="solver_ssz" localSheetId="2" hidden="1">100</definedName>
     <definedName name="solver_tim" localSheetId="1" hidden="1">2147483647</definedName>
-    <definedName name="solver_tim" localSheetId="2" hidden="1">2147483647</definedName>
     <definedName name="solver_tol" localSheetId="1" hidden="1">0.01</definedName>
-    <definedName name="solver_tol" localSheetId="2" hidden="1">0.01</definedName>
     <definedName name="solver_typ" localSheetId="1" hidden="1">1</definedName>
-    <definedName name="solver_typ" localSheetId="2" hidden="1">1</definedName>
     <definedName name="solver_val" localSheetId="1" hidden="1">0</definedName>
-    <definedName name="solver_val" localSheetId="2" hidden="1">0</definedName>
     <definedName name="solver_ver" localSheetId="1" hidden="1">3</definedName>
-    <definedName name="solver_ver" localSheetId="2" hidden="1">3</definedName>
     <definedName name="TempHoursPerWorker">Inputs!$B$16</definedName>
     <definedName name="TempLaborCapacity">Calc!$B$17</definedName>
     <definedName name="TempLaborHoursUsed">Calc!$B$16</definedName>
@@ -399,11 +359,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="4">
+    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="\$#,##0"/>
-    <numFmt numFmtId="166" formatCode="\$#,##0.00"/>
+    <numFmt numFmtId="165" formatCode="\$#,##0.00"/>
+    <numFmt numFmtId="167" formatCode="_(* #,##0.0000_);_(* \(#,##0.0000\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -416,6 +378,13 @@
       <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -435,15 +404,15 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="4" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -451,9 +420,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -811,7 +782,7 @@
       <c r="E5" s="3">
         <v>880</v>
       </c>
-      <c r="F5" s="4">
+      <c r="F5" s="10">
         <v>0.1</v>
       </c>
     </row>
@@ -832,7 +803,7 @@
       <c r="E6" s="3">
         <v>440</v>
       </c>
-      <c r="F6" s="4">
+      <c r="F6" s="10">
         <v>2.5000000000000001E-2</v>
       </c>
     </row>
@@ -852,7 +823,7 @@
       <c r="E7" s="3">
         <v>880</v>
       </c>
-      <c r="F7" s="4">
+      <c r="F7" s="10">
         <v>1.2500000000000001E-2</v>
       </c>
     </row>
@@ -873,7 +844,7 @@
       <c r="A11" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B11" s="5">
+      <c r="B11" s="4">
         <v>20000</v>
       </c>
     </row>
@@ -1030,7 +1001,7 @@
       <c r="A12" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B12" s="6">
+      <c r="B12" s="5">
         <f>LaborHoursTomatoes+LaborHoursCarrots+LaborHoursMesclun</f>
         <v>5277.2161142738878</v>
       </c>
@@ -1071,7 +1042,7 @@
       <c r="A18" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B18" s="7">
+      <c r="B18" s="6">
         <f>OwnLaborHoursUsed*OwnWageRate+TempLaborHoursUsed*TempWageRate</f>
         <v>104118.335317255</v>
       </c>
@@ -1085,7 +1056,7 @@
       <c r="A21" t="s">
         <v>40</v>
       </c>
-      <c r="B21" s="5">
+      <c r="B21" s="4">
         <f>BedsTomatoes*RevenuePerBedTomatoes+BedsCarrots*RevenuePerBedCarrots+BedsMesclun*RevenuePerBedMesclun</f>
         <v>210880</v>
       </c>
@@ -1094,7 +1065,7 @@
       <c r="A22" t="s">
         <v>41</v>
       </c>
-      <c r="B22" s="5">
+      <c r="B22" s="4">
         <f>BedsTomatoes*FertilizerPerBedTomatoes+BedsCarrots*FertilizerPerBedCarrots+BedsMesclun*FertilizerPerBedMesclun</f>
         <v>44000</v>
       </c>
@@ -1103,7 +1074,7 @@
       <c r="A23" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="B23" s="7">
+      <c r="B23" s="6">
         <f>FixedCosts+FertilizerCost+LaborCost</f>
         <v>168118.335317255</v>
       </c>
@@ -1112,7 +1083,7 @@
       <c r="A24" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="B24" s="10">
+      <c r="B24" s="9">
         <f>Revenue-TotalCost</f>
         <v>42761.664682745002</v>
       </c>
@@ -1254,7 +1225,7 @@
       <c r="A14" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="B14" s="9" t="s">
+      <c r="B14" s="8" t="s">
         <v>72</v>
       </c>
     </row>
@@ -1302,7 +1273,7 @@
       <c r="A21" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="B21" s="8">
+      <c r="B21" s="7">
         <f>TotalBedsPlanted</f>
         <v>60</v>
       </c>
@@ -1320,7 +1291,7 @@
       <c r="A23" t="s">
         <v>40</v>
       </c>
-      <c r="B23" s="5">
+      <c r="B23" s="4">
         <f>Revenue</f>
         <v>210880</v>
       </c>
@@ -1329,7 +1300,7 @@
       <c r="A24" t="s">
         <v>42</v>
       </c>
-      <c r="B24" s="5">
+      <c r="B24" s="4">
         <f>TotalCost</f>
         <v>168118.335317255</v>
       </c>
@@ -1338,7 +1309,7 @@
       <c r="A25" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="B25" s="7">
+      <c r="B25" s="6">
         <f>Profit</f>
         <v>42761.664682745002</v>
       </c>

</xml_diff>

<commit_message>
fixed chart axis title overlap in MC Schedule
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UuHPa2K2Y6ovJRTQQ5rXcP
</commit_message>
<xml_diff>
--- a/capabilities/marginal-analysis/model.xlsx
+++ b/capabilities/marginal-analysis/model.xlsx
@@ -268,6 +268,7 @@
           </a:p>
         </rich>
       </tx>
+      <overlay val="0"/>
     </title>
     <plotArea>
       <lineChart>
@@ -380,11 +381,11 @@
           <orientation val="minMax"/>
         </scaling>
         <delete val="0"/>
-        <axPos val="l"/>
+        <axPos val="b"/>
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
+              <a:bodyPr rot="0" vert="horz"/>
               <a:p>
                 <a:pPr>
                   <a:defRPr/>
@@ -395,9 +396,11 @@
               </a:p>
             </rich>
           </tx>
+          <overlay val="0"/>
         </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
+        <tickLblPos val="nextTo"/>
         <crossAx val="100"/>
         <lblOffset val="100"/>
       </catAx>
@@ -412,7 +415,7 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
+              <a:bodyPr rot="-5400000" vert="horz"/>
               <a:p>
                 <a:pPr>
                   <a:defRPr/>
@@ -423,15 +426,18 @@
               </a:p>
             </rich>
           </tx>
+          <overlay val="0"/>
         </title>
         <numFmt formatCode="\$#,##0" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
+        <tickLblPos val="nextTo"/>
         <crossAx val="10"/>
       </valAx>
     </plotArea>
     <legend>
-      <legendPos val="r"/>
+      <legendPos val="b"/>
+      <overlay val="0"/>
     </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
@@ -456,6 +462,7 @@
           </a:p>
         </rich>
       </tx>
+      <overlay val="0"/>
     </title>
     <plotArea>
       <lineChart>
@@ -568,11 +575,11 @@
           <orientation val="minMax"/>
         </scaling>
         <delete val="0"/>
-        <axPos val="l"/>
+        <axPos val="b"/>
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
+              <a:bodyPr rot="0" vert="horz"/>
               <a:p>
                 <a:pPr>
                   <a:defRPr/>
@@ -583,9 +590,11 @@
               </a:p>
             </rich>
           </tx>
+          <overlay val="0"/>
         </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
+        <tickLblPos val="nextTo"/>
         <crossAx val="100"/>
         <lblOffset val="100"/>
       </catAx>
@@ -600,7 +609,7 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
+              <a:bodyPr rot="-5400000" vert="horz"/>
               <a:p>
                 <a:pPr>
                   <a:defRPr/>
@@ -611,15 +620,18 @@
               </a:p>
             </rich>
           </tx>
+          <overlay val="0"/>
         </title>
         <numFmt formatCode="\$#,##0" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
+        <tickLblPos val="nextTo"/>
         <crossAx val="10"/>
       </valAx>
     </plotArea>
     <legend>
-      <legendPos val="r"/>
+      <legendPos val="b"/>
+      <overlay val="0"/>
     </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
@@ -644,6 +656,7 @@
           </a:p>
         </rich>
       </tx>
+      <overlay val="0"/>
     </title>
     <plotArea>
       <lineChart>
@@ -756,11 +769,11 @@
           <orientation val="minMax"/>
         </scaling>
         <delete val="0"/>
-        <axPos val="l"/>
+        <axPos val="b"/>
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
+              <a:bodyPr rot="0" vert="horz"/>
               <a:p>
                 <a:pPr>
                   <a:defRPr/>
@@ -771,9 +784,11 @@
               </a:p>
             </rich>
           </tx>
+          <overlay val="0"/>
         </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
+        <tickLblPos val="nextTo"/>
         <crossAx val="100"/>
         <lblOffset val="100"/>
       </catAx>
@@ -788,7 +803,7 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
+              <a:bodyPr rot="-5400000" vert="horz"/>
               <a:p>
                 <a:pPr>
                   <a:defRPr/>
@@ -799,15 +814,18 @@
               </a:p>
             </rich>
           </tx>
+          <overlay val="0"/>
         </title>
         <numFmt formatCode="\$#,##0" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
+        <tickLblPos val="nextTo"/>
         <crossAx val="10"/>
       </valAx>
     </plotArea>
     <legend>
-      <legendPos val="r"/>
+      <legendPos val="b"/>
+      <overlay val="0"/>
     </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>

</xml_diff>

<commit_message>
added in-mix MC column and beyond-cap rows to MC Schedule
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UuHPa2K2Y6ovJRTQQ5rXcP
</commit_message>
<xml_diff>
--- a/capabilities/marginal-analysis/model.xlsx
+++ b/capabilities/marginal-analysis/model.xlsx
@@ -112,7 +112,7 @@
     <numFmt numFmtId="165" formatCode="\$#,##0.00"/>
     <numFmt numFmtId="166" formatCode="_(* #,##0.0000_);_(* \(#,##0.0000\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -136,6 +136,10 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00808080"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -158,7 +162,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -174,6 +178,9 @@
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -263,7 +270,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Tomatoes: MC vs price (standalone)</a:t>
+              <a:t>Tomatoes: MC vs price</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -372,6 +379,39 @@
           </val>
           <smooth val="0"/>
         </ser>
+        <ser>
+          <idx val="3"/>
+          <order val="3"/>
+          <tx>
+            <strRef>
+              <f>'MC Schedule'!K8</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'MC Schedule'!$A$10:$A$29</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'MC Schedule'!$K$10:$K$29</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
         <axId val="10"/>
         <axId val="100"/>
       </lineChart>
@@ -403,6 +443,7 @@
         <tickLblPos val="nextTo"/>
         <crossAx val="100"/>
         <lblOffset val="100"/>
+        <tickLblSkip val="1"/>
       </catAx>
       <valAx>
         <axId val="100"/>
@@ -457,7 +498,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Carrots: MC vs price (standalone)</a:t>
+              <a:t>Carrots: MC vs price</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -566,6 +607,39 @@
           </val>
           <smooth val="0"/>
         </ser>
+        <ser>
+          <idx val="3"/>
+          <order val="3"/>
+          <tx>
+            <strRef>
+              <f>'MC Schedule'!K33</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'MC Schedule'!$A$35:$A$54</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'MC Schedule'!$K$35:$K$54</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
         <axId val="10"/>
         <axId val="100"/>
       </lineChart>
@@ -597,6 +671,7 @@
         <tickLblPos val="nextTo"/>
         <crossAx val="100"/>
         <lblOffset val="100"/>
+        <tickLblSkip val="1"/>
       </catAx>
       <valAx>
         <axId val="100"/>
@@ -651,7 +726,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Mesclun: MC vs price (standalone)</a:t>
+              <a:t>Mesclun: MC vs price</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -666,7 +741,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'MC Schedule'!F58</f>
+              <f>'MC Schedule'!F62</f>
             </strRef>
           </tx>
           <spPr>
@@ -684,12 +759,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'MC Schedule'!$A$60:$A$89</f>
+              <f>'MC Schedule'!$A$64:$A$93</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'MC Schedule'!$F$60:$F$89</f>
+              <f>'MC Schedule'!$F$64:$F$93</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -699,7 +774,7 @@
           <order val="1"/>
           <tx>
             <strRef>
-              <f>'MC Schedule'!G58</f>
+              <f>'MC Schedule'!G62</f>
             </strRef>
           </tx>
           <spPr>
@@ -717,12 +792,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'MC Schedule'!$A$60:$A$89</f>
+              <f>'MC Schedule'!$A$64:$A$93</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'MC Schedule'!$G$60:$G$89</f>
+              <f>'MC Schedule'!$G$64:$G$93</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -732,7 +807,7 @@
           <order val="2"/>
           <tx>
             <strRef>
-              <f>'MC Schedule'!H58</f>
+              <f>'MC Schedule'!H62</f>
             </strRef>
           </tx>
           <spPr>
@@ -750,12 +825,45 @@
           </marker>
           <cat>
             <numRef>
-              <f>'MC Schedule'!$A$60:$A$89</f>
+              <f>'MC Schedule'!$A$64:$A$93</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'MC Schedule'!$H$60:$H$89</f>
+              <f>'MC Schedule'!$H$64:$H$93</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="3"/>
+          <order val="3"/>
+          <tx>
+            <strRef>
+              <f>'MC Schedule'!K62</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'MC Schedule'!$A$64:$A$93</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'MC Schedule'!$K$64:$K$93</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -791,6 +899,7 @@
         <tickLblPos val="nextTo"/>
         <crossAx val="100"/>
         <lblOffset val="100"/>
+        <tickLblSkip val="1"/>
       </catAx>
       <valAx>
         <axId val="100"/>
@@ -837,7 +946,7 @@
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>11</col>
+      <col>12</col>
       <colOff>0</colOff>
       <row>6</row>
       <rowOff>0</rowOff>
@@ -859,7 +968,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>11</col>
+      <col>12</col>
       <colOff>0</colOff>
       <row>26</row>
       <rowOff>0</rowOff>
@@ -881,12 +990,12 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>11</col>
+      <col>12</col>
       <colOff>0</colOff>
       <row>46</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6120000" cy="3240000"/>
+    <ext cx="7920000" cy="3240000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="3" name="Chart 3"/>
@@ -1969,7 +2078,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J89"/>
+  <dimension ref="A1:K97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1982,6 +2091,7 @@
     <col width="15" customWidth="1" min="8" max="8"/>
     <col width="15" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="17" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2008,7 +2118,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>At the solved mix (Calc), total labor is far past OwnLaborHours, so every marginal hour there is paid at TempWageRate.</t>
+          <t>MC in solved mix = the same bed added to the mix on Calc: the other two crops stay at their Calc bed counts, so the wage on each marginal hour depends on total farm labor, not this crop alone.</t>
         </is>
       </c>
     </row>
@@ -2019,6 +2129,13 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Rows in grey italics are past the crop's MaxBeds: what one more bed would earn if the cap were relaxed (the value of relaxing it). Charts stop at the cap.</t>
+        </is>
+      </c>
+    </row>
     <row r="7">
       <c r="A7" s="12" t="inlineStr">
         <is>
@@ -2054,7 +2171,7 @@
       </c>
       <c r="F8" s="12" t="inlineStr">
         <is>
-          <t>MC</t>
+          <t>MC standalone</t>
         </is>
       </c>
       <c r="G8" s="12" t="inlineStr">
@@ -2075,6 +2192,11 @@
       <c r="J8" s="12" t="inlineStr">
         <is>
           <t>Standalone profit</t>
+        </is>
+      </c>
+      <c r="K8" s="12" t="inlineStr">
+        <is>
+          <t>MC in solved mix</t>
         </is>
       </c>
     </row>
@@ -2098,12 +2220,8 @@
         <f>C9+D9</f>
         <v/>
       </c>
-      <c r="H9" s="4">
-        <f>RevenuePerBedTomatoes</f>
-        <v/>
-      </c>
       <c r="J9" s="4">
-        <f>A9*H9-E9-FixedCosts</f>
+        <f>A9*RevenuePerBedTomatoes-E9-FixedCosts</f>
         <v/>
       </c>
     </row>
@@ -2144,7 +2262,11 @@
         <v/>
       </c>
       <c r="J10" s="4">
-        <f>A10*H10-E10-FixedCosts</f>
+        <f>A10*RevenuePerBedTomatoes-E10-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K10" s="4">
+        <f>(MIN(((TotalLaborHours-LaborHoursTomatoes)+B10),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursTomatoes)+B10)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursTomatoes)+B9),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursTomatoes)+B9)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedTomatoes</f>
         <v/>
       </c>
     </row>
@@ -2185,7 +2307,11 @@
         <v/>
       </c>
       <c r="J11" s="4">
-        <f>A11*H11-E11-FixedCosts</f>
+        <f>A11*RevenuePerBedTomatoes-E11-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K11" s="4">
+        <f>(MIN(((TotalLaborHours-LaborHoursTomatoes)+B11),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursTomatoes)+B11)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursTomatoes)+B10),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursTomatoes)+B10)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedTomatoes</f>
         <v/>
       </c>
     </row>
@@ -2226,7 +2352,11 @@
         <v/>
       </c>
       <c r="J12" s="4">
-        <f>A12*H12-E12-FixedCosts</f>
+        <f>A12*RevenuePerBedTomatoes-E12-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K12" s="4">
+        <f>(MIN(((TotalLaborHours-LaborHoursTomatoes)+B12),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursTomatoes)+B12)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursTomatoes)+B11),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursTomatoes)+B11)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedTomatoes</f>
         <v/>
       </c>
     </row>
@@ -2267,7 +2397,11 @@
         <v/>
       </c>
       <c r="J13" s="4">
-        <f>A13*H13-E13-FixedCosts</f>
+        <f>A13*RevenuePerBedTomatoes-E13-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K13" s="4">
+        <f>(MIN(((TotalLaborHours-LaborHoursTomatoes)+B13),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursTomatoes)+B13)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursTomatoes)+B12),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursTomatoes)+B12)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedTomatoes</f>
         <v/>
       </c>
     </row>
@@ -2308,7 +2442,11 @@
         <v/>
       </c>
       <c r="J14" s="4">
-        <f>A14*H14-E14-FixedCosts</f>
+        <f>A14*RevenuePerBedTomatoes-E14-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K14" s="4">
+        <f>(MIN(((TotalLaborHours-LaborHoursTomatoes)+B14),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursTomatoes)+B14)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursTomatoes)+B13),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursTomatoes)+B13)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedTomatoes</f>
         <v/>
       </c>
     </row>
@@ -2349,7 +2487,11 @@
         <v/>
       </c>
       <c r="J15" s="4">
-        <f>A15*H15-E15-FixedCosts</f>
+        <f>A15*RevenuePerBedTomatoes-E15-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K15" s="4">
+        <f>(MIN(((TotalLaborHours-LaborHoursTomatoes)+B15),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursTomatoes)+B15)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursTomatoes)+B14),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursTomatoes)+B14)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedTomatoes</f>
         <v/>
       </c>
     </row>
@@ -2390,7 +2532,11 @@
         <v/>
       </c>
       <c r="J16" s="4">
-        <f>A16*H16-E16-FixedCosts</f>
+        <f>A16*RevenuePerBedTomatoes-E16-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K16" s="4">
+        <f>(MIN(((TotalLaborHours-LaborHoursTomatoes)+B16),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursTomatoes)+B16)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursTomatoes)+B15),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursTomatoes)+B15)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedTomatoes</f>
         <v/>
       </c>
     </row>
@@ -2431,7 +2577,11 @@
         <v/>
       </c>
       <c r="J17" s="4">
-        <f>A17*H17-E17-FixedCosts</f>
+        <f>A17*RevenuePerBedTomatoes-E17-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K17" s="4">
+        <f>(MIN(((TotalLaborHours-LaborHoursTomatoes)+B17),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursTomatoes)+B17)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursTomatoes)+B16),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursTomatoes)+B16)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedTomatoes</f>
         <v/>
       </c>
     </row>
@@ -2472,7 +2622,11 @@
         <v/>
       </c>
       <c r="J18" s="4">
-        <f>A18*H18-E18-FixedCosts</f>
+        <f>A18*RevenuePerBedTomatoes-E18-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K18" s="4">
+        <f>(MIN(((TotalLaborHours-LaborHoursTomatoes)+B18),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursTomatoes)+B18)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursTomatoes)+B17),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursTomatoes)+B17)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedTomatoes</f>
         <v/>
       </c>
     </row>
@@ -2513,7 +2667,11 @@
         <v/>
       </c>
       <c r="J19" s="4">
-        <f>A19*H19-E19-FixedCosts</f>
+        <f>A19*RevenuePerBedTomatoes-E19-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K19" s="4">
+        <f>(MIN(((TotalLaborHours-LaborHoursTomatoes)+B19),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursTomatoes)+B19)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursTomatoes)+B18),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursTomatoes)+B18)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedTomatoes</f>
         <v/>
       </c>
     </row>
@@ -2554,7 +2712,11 @@
         <v/>
       </c>
       <c r="J20" s="4">
-        <f>A20*H20-E20-FixedCosts</f>
+        <f>A20*RevenuePerBedTomatoes-E20-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K20" s="4">
+        <f>(MIN(((TotalLaborHours-LaborHoursTomatoes)+B20),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursTomatoes)+B20)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursTomatoes)+B19),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursTomatoes)+B19)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedTomatoes</f>
         <v/>
       </c>
     </row>
@@ -2595,7 +2757,11 @@
         <v/>
       </c>
       <c r="J21" s="4">
-        <f>A21*H21-E21-FixedCosts</f>
+        <f>A21*RevenuePerBedTomatoes-E21-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K21" s="4">
+        <f>(MIN(((TotalLaborHours-LaborHoursTomatoes)+B21),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursTomatoes)+B21)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursTomatoes)+B20),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursTomatoes)+B20)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedTomatoes</f>
         <v/>
       </c>
     </row>
@@ -2636,7 +2802,11 @@
         <v/>
       </c>
       <c r="J22" s="4">
-        <f>A22*H22-E22-FixedCosts</f>
+        <f>A22*RevenuePerBedTomatoes-E22-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K22" s="4">
+        <f>(MIN(((TotalLaborHours-LaborHoursTomatoes)+B22),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursTomatoes)+B22)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursTomatoes)+B21),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursTomatoes)+B21)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedTomatoes</f>
         <v/>
       </c>
     </row>
@@ -2677,7 +2847,11 @@
         <v/>
       </c>
       <c r="J23" s="4">
-        <f>A23*H23-E23-FixedCosts</f>
+        <f>A23*RevenuePerBedTomatoes-E23-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K23" s="4">
+        <f>(MIN(((TotalLaborHours-LaborHoursTomatoes)+B23),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursTomatoes)+B23)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursTomatoes)+B22),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursTomatoes)+B22)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedTomatoes</f>
         <v/>
       </c>
     </row>
@@ -2718,7 +2892,11 @@
         <v/>
       </c>
       <c r="J24" s="4">
-        <f>A24*H24-E24-FixedCosts</f>
+        <f>A24*RevenuePerBedTomatoes-E24-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K24" s="4">
+        <f>(MIN(((TotalLaborHours-LaborHoursTomatoes)+B24),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursTomatoes)+B24)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursTomatoes)+B23),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursTomatoes)+B23)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedTomatoes</f>
         <v/>
       </c>
     </row>
@@ -2759,7 +2937,11 @@
         <v/>
       </c>
       <c r="J25" s="4">
-        <f>A25*H25-E25-FixedCosts</f>
+        <f>A25*RevenuePerBedTomatoes-E25-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K25" s="4">
+        <f>(MIN(((TotalLaborHours-LaborHoursTomatoes)+B25),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursTomatoes)+B25)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursTomatoes)+B24),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursTomatoes)+B24)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedTomatoes</f>
         <v/>
       </c>
     </row>
@@ -2800,7 +2982,11 @@
         <v/>
       </c>
       <c r="J26" s="4">
-        <f>A26*H26-E26-FixedCosts</f>
+        <f>A26*RevenuePerBedTomatoes-E26-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K26" s="4">
+        <f>(MIN(((TotalLaborHours-LaborHoursTomatoes)+B26),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursTomatoes)+B26)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursTomatoes)+B25),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursTomatoes)+B25)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedTomatoes</f>
         <v/>
       </c>
     </row>
@@ -2841,7 +3027,11 @@
         <v/>
       </c>
       <c r="J27" s="4">
-        <f>A27*H27-E27-FixedCosts</f>
+        <f>A27*RevenuePerBedTomatoes-E27-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K27" s="4">
+        <f>(MIN(((TotalLaborHours-LaborHoursTomatoes)+B27),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursTomatoes)+B27)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursTomatoes)+B26),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursTomatoes)+B26)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedTomatoes</f>
         <v/>
       </c>
     </row>
@@ -2882,7 +3072,11 @@
         <v/>
       </c>
       <c r="J28" s="4">
-        <f>A28*H28-E28-FixedCosts</f>
+        <f>A28*RevenuePerBedTomatoes-E28-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K28" s="4">
+        <f>(MIN(((TotalLaborHours-LaborHoursTomatoes)+B28),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursTomatoes)+B28)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursTomatoes)+B27),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursTomatoes)+B27)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedTomatoes</f>
         <v/>
       </c>
     </row>
@@ -2923,7 +3117,11 @@
         <v/>
       </c>
       <c r="J29" s="4">
-        <f>A29*H29-E29-FixedCosts</f>
+        <f>A29*RevenuePerBedTomatoes-E29-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K29" s="4">
+        <f>(MIN(((TotalLaborHours-LaborHoursTomatoes)+B29),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursTomatoes)+B29)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursTomatoes)+B28),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursTomatoes)+B28)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedTomatoes</f>
         <v/>
       </c>
     </row>
@@ -2962,7 +3160,7 @@
       </c>
       <c r="F33" s="12" t="inlineStr">
         <is>
-          <t>MC</t>
+          <t>MC standalone</t>
         </is>
       </c>
       <c r="G33" s="12" t="inlineStr">
@@ -2983,6 +3181,11 @@
       <c r="J33" s="12" t="inlineStr">
         <is>
           <t>Standalone profit</t>
+        </is>
+      </c>
+      <c r="K33" s="12" t="inlineStr">
+        <is>
+          <t>MC in solved mix</t>
         </is>
       </c>
     </row>
@@ -3006,12 +3209,8 @@
         <f>C34+D34</f>
         <v/>
       </c>
-      <c r="H34" s="4">
-        <f>RevenuePerBedCarrots</f>
-        <v/>
-      </c>
       <c r="J34" s="4">
-        <f>A34*H34-E34-FixedCosts</f>
+        <f>A34*RevenuePerBedCarrots-E34-FixedCosts</f>
         <v/>
       </c>
     </row>
@@ -3052,7 +3251,11 @@
         <v/>
       </c>
       <c r="J35" s="4">
-        <f>A35*H35-E35-FixedCosts</f>
+        <f>A35*RevenuePerBedCarrots-E35-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K35" s="4">
+        <f>(MIN(((TotalLaborHours-LaborHoursCarrots)+B35),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursCarrots)+B35)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursCarrots)+B34),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursCarrots)+B34)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedCarrots</f>
         <v/>
       </c>
     </row>
@@ -3093,7 +3296,11 @@
         <v/>
       </c>
       <c r="J36" s="4">
-        <f>A36*H36-E36-FixedCosts</f>
+        <f>A36*RevenuePerBedCarrots-E36-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K36" s="4">
+        <f>(MIN(((TotalLaborHours-LaborHoursCarrots)+B36),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursCarrots)+B36)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursCarrots)+B35),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursCarrots)+B35)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedCarrots</f>
         <v/>
       </c>
     </row>
@@ -3134,7 +3341,11 @@
         <v/>
       </c>
       <c r="J37" s="4">
-        <f>A37*H37-E37-FixedCosts</f>
+        <f>A37*RevenuePerBedCarrots-E37-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K37" s="4">
+        <f>(MIN(((TotalLaborHours-LaborHoursCarrots)+B37),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursCarrots)+B37)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursCarrots)+B36),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursCarrots)+B36)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedCarrots</f>
         <v/>
       </c>
     </row>
@@ -3175,7 +3386,11 @@
         <v/>
       </c>
       <c r="J38" s="4">
-        <f>A38*H38-E38-FixedCosts</f>
+        <f>A38*RevenuePerBedCarrots-E38-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K38" s="4">
+        <f>(MIN(((TotalLaborHours-LaborHoursCarrots)+B38),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursCarrots)+B38)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursCarrots)+B37),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursCarrots)+B37)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedCarrots</f>
         <v/>
       </c>
     </row>
@@ -3216,7 +3431,11 @@
         <v/>
       </c>
       <c r="J39" s="4">
-        <f>A39*H39-E39-FixedCosts</f>
+        <f>A39*RevenuePerBedCarrots-E39-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K39" s="4">
+        <f>(MIN(((TotalLaborHours-LaborHoursCarrots)+B39),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursCarrots)+B39)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursCarrots)+B38),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursCarrots)+B38)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedCarrots</f>
         <v/>
       </c>
     </row>
@@ -3257,7 +3476,11 @@
         <v/>
       </c>
       <c r="J40" s="4">
-        <f>A40*H40-E40-FixedCosts</f>
+        <f>A40*RevenuePerBedCarrots-E40-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K40" s="4">
+        <f>(MIN(((TotalLaborHours-LaborHoursCarrots)+B40),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursCarrots)+B40)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursCarrots)+B39),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursCarrots)+B39)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedCarrots</f>
         <v/>
       </c>
     </row>
@@ -3298,7 +3521,11 @@
         <v/>
       </c>
       <c r="J41" s="4">
-        <f>A41*H41-E41-FixedCosts</f>
+        <f>A41*RevenuePerBedCarrots-E41-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K41" s="4">
+        <f>(MIN(((TotalLaborHours-LaborHoursCarrots)+B41),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursCarrots)+B41)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursCarrots)+B40),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursCarrots)+B40)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedCarrots</f>
         <v/>
       </c>
     </row>
@@ -3339,7 +3566,11 @@
         <v/>
       </c>
       <c r="J42" s="4">
-        <f>A42*H42-E42-FixedCosts</f>
+        <f>A42*RevenuePerBedCarrots-E42-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K42" s="4">
+        <f>(MIN(((TotalLaborHours-LaborHoursCarrots)+B42),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursCarrots)+B42)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursCarrots)+B41),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursCarrots)+B41)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedCarrots</f>
         <v/>
       </c>
     </row>
@@ -3380,7 +3611,11 @@
         <v/>
       </c>
       <c r="J43" s="4">
-        <f>A43*H43-E43-FixedCosts</f>
+        <f>A43*RevenuePerBedCarrots-E43-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K43" s="4">
+        <f>(MIN(((TotalLaborHours-LaborHoursCarrots)+B43),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursCarrots)+B43)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursCarrots)+B42),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursCarrots)+B42)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedCarrots</f>
         <v/>
       </c>
     </row>
@@ -3421,7 +3656,11 @@
         <v/>
       </c>
       <c r="J44" s="4">
-        <f>A44*H44-E44-FixedCosts</f>
+        <f>A44*RevenuePerBedCarrots-E44-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K44" s="4">
+        <f>(MIN(((TotalLaborHours-LaborHoursCarrots)+B44),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursCarrots)+B44)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursCarrots)+B43),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursCarrots)+B43)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedCarrots</f>
         <v/>
       </c>
     </row>
@@ -3462,7 +3701,11 @@
         <v/>
       </c>
       <c r="J45" s="4">
-        <f>A45*H45-E45-FixedCosts</f>
+        <f>A45*RevenuePerBedCarrots-E45-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K45" s="4">
+        <f>(MIN(((TotalLaborHours-LaborHoursCarrots)+B45),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursCarrots)+B45)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursCarrots)+B44),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursCarrots)+B44)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedCarrots</f>
         <v/>
       </c>
     </row>
@@ -3503,7 +3746,11 @@
         <v/>
       </c>
       <c r="J46" s="4">
-        <f>A46*H46-E46-FixedCosts</f>
+        <f>A46*RevenuePerBedCarrots-E46-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K46" s="4">
+        <f>(MIN(((TotalLaborHours-LaborHoursCarrots)+B46),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursCarrots)+B46)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursCarrots)+B45),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursCarrots)+B45)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedCarrots</f>
         <v/>
       </c>
     </row>
@@ -3544,7 +3791,11 @@
         <v/>
       </c>
       <c r="J47" s="4">
-        <f>A47*H47-E47-FixedCosts</f>
+        <f>A47*RevenuePerBedCarrots-E47-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K47" s="4">
+        <f>(MIN(((TotalLaborHours-LaborHoursCarrots)+B47),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursCarrots)+B47)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursCarrots)+B46),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursCarrots)+B46)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedCarrots</f>
         <v/>
       </c>
     </row>
@@ -3585,7 +3836,11 @@
         <v/>
       </c>
       <c r="J48" s="4">
-        <f>A48*H48-E48-FixedCosts</f>
+        <f>A48*RevenuePerBedCarrots-E48-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K48" s="4">
+        <f>(MIN(((TotalLaborHours-LaborHoursCarrots)+B48),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursCarrots)+B48)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursCarrots)+B47),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursCarrots)+B47)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedCarrots</f>
         <v/>
       </c>
     </row>
@@ -3626,7 +3881,11 @@
         <v/>
       </c>
       <c r="J49" s="4">
-        <f>A49*H49-E49-FixedCosts</f>
+        <f>A49*RevenuePerBedCarrots-E49-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K49" s="4">
+        <f>(MIN(((TotalLaborHours-LaborHoursCarrots)+B49),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursCarrots)+B49)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursCarrots)+B48),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursCarrots)+B48)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedCarrots</f>
         <v/>
       </c>
     </row>
@@ -3667,7 +3926,11 @@
         <v/>
       </c>
       <c r="J50" s="4">
-        <f>A50*H50-E50-FixedCosts</f>
+        <f>A50*RevenuePerBedCarrots-E50-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K50" s="4">
+        <f>(MIN(((TotalLaborHours-LaborHoursCarrots)+B50),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursCarrots)+B50)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursCarrots)+B49),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursCarrots)+B49)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedCarrots</f>
         <v/>
       </c>
     </row>
@@ -3708,7 +3971,11 @@
         <v/>
       </c>
       <c r="J51" s="4">
-        <f>A51*H51-E51-FixedCosts</f>
+        <f>A51*RevenuePerBedCarrots-E51-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K51" s="4">
+        <f>(MIN(((TotalLaborHours-LaborHoursCarrots)+B51),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursCarrots)+B51)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursCarrots)+B50),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursCarrots)+B50)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedCarrots</f>
         <v/>
       </c>
     </row>
@@ -3749,7 +4016,11 @@
         <v/>
       </c>
       <c r="J52" s="4">
-        <f>A52*H52-E52-FixedCosts</f>
+        <f>A52*RevenuePerBedCarrots-E52-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K52" s="4">
+        <f>(MIN(((TotalLaborHours-LaborHoursCarrots)+B52),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursCarrots)+B52)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursCarrots)+B51),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursCarrots)+B51)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedCarrots</f>
         <v/>
       </c>
     </row>
@@ -3790,7 +4061,11 @@
         <v/>
       </c>
       <c r="J53" s="4">
-        <f>A53*H53-E53-FixedCosts</f>
+        <f>A53*RevenuePerBedCarrots-E53-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K53" s="4">
+        <f>(MIN(((TotalLaborHours-LaborHoursCarrots)+B53),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursCarrots)+B53)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursCarrots)+B52),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursCarrots)+B52)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedCarrots</f>
         <v/>
       </c>
     </row>
@@ -3831,224 +4106,261 @@
         <v/>
       </c>
       <c r="J54" s="4">
-        <f>A54*H54-E54-FixedCosts</f>
+        <f>A54*RevenuePerBedCarrots-E54-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K54" s="4">
+        <f>(MIN(((TotalLaborHours-LaborHoursCarrots)+B54),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursCarrots)+B54)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursCarrots)+B53),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursCarrots)+B53)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedCarrots</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="13" t="n">
+        <v>21</v>
+      </c>
+      <c r="B55" s="14">
+        <f>A55*LaborHrsPerBedCarrots*SeasonWeeks*(1+DimReturnsCarrots)^A55</f>
+        <v/>
+      </c>
+      <c r="C55" s="15">
+        <f>MIN(B55,OwnLaborHours)*OwnWageRate+MAX(B55-OwnLaborHours,0)*TempWageRate</f>
+        <v/>
+      </c>
+      <c r="D55" s="15">
+        <f>A55*FertilizerPerBedCarrots</f>
+        <v/>
+      </c>
+      <c r="E55" s="15">
+        <f>C55+D55</f>
+        <v/>
+      </c>
+      <c r="F55" s="15">
+        <f>E55-E54</f>
+        <v/>
+      </c>
+      <c r="G55" s="15">
+        <f>E55/A55</f>
+        <v/>
+      </c>
+      <c r="H55" s="15">
+        <f>RevenuePerBedCarrots</f>
+        <v/>
+      </c>
+      <c r="I55" s="15">
+        <f>H55-F55</f>
+        <v/>
+      </c>
+      <c r="J55" s="15">
+        <f>A55*RevenuePerBedCarrots-E55-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K55" s="15">
+        <f>(MIN(((TotalLaborHours-LaborHoursCarrots)+B55),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursCarrots)+B55)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursCarrots)+B54),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursCarrots)+B54)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedCarrots</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="13" t="n">
+        <v>22</v>
+      </c>
+      <c r="B56" s="14">
+        <f>A56*LaborHrsPerBedCarrots*SeasonWeeks*(1+DimReturnsCarrots)^A56</f>
+        <v/>
+      </c>
+      <c r="C56" s="15">
+        <f>MIN(B56,OwnLaborHours)*OwnWageRate+MAX(B56-OwnLaborHours,0)*TempWageRate</f>
+        <v/>
+      </c>
+      <c r="D56" s="15">
+        <f>A56*FertilizerPerBedCarrots</f>
+        <v/>
+      </c>
+      <c r="E56" s="15">
+        <f>C56+D56</f>
+        <v/>
+      </c>
+      <c r="F56" s="15">
+        <f>E56-E55</f>
+        <v/>
+      </c>
+      <c r="G56" s="15">
+        <f>E56/A56</f>
+        <v/>
+      </c>
+      <c r="H56" s="15">
+        <f>RevenuePerBedCarrots</f>
+        <v/>
+      </c>
+      <c r="I56" s="15">
+        <f>H56-F56</f>
+        <v/>
+      </c>
+      <c r="J56" s="15">
+        <f>A56*RevenuePerBedCarrots-E56-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K56" s="15">
+        <f>(MIN(((TotalLaborHours-LaborHoursCarrots)+B56),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursCarrots)+B56)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursCarrots)+B55),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursCarrots)+B55)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedCarrots</f>
         <v/>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="12" t="inlineStr">
+      <c r="A57" s="13" t="n">
+        <v>23</v>
+      </c>
+      <c r="B57" s="14">
+        <f>A57*LaborHrsPerBedCarrots*SeasonWeeks*(1+DimReturnsCarrots)^A57</f>
+        <v/>
+      </c>
+      <c r="C57" s="15">
+        <f>MIN(B57,OwnLaborHours)*OwnWageRate+MAX(B57-OwnLaborHours,0)*TempWageRate</f>
+        <v/>
+      </c>
+      <c r="D57" s="15">
+        <f>A57*FertilizerPerBedCarrots</f>
+        <v/>
+      </c>
+      <c r="E57" s="15">
+        <f>C57+D57</f>
+        <v/>
+      </c>
+      <c r="F57" s="15">
+        <f>E57-E56</f>
+        <v/>
+      </c>
+      <c r="G57" s="15">
+        <f>E57/A57</f>
+        <v/>
+      </c>
+      <c r="H57" s="15">
+        <f>RevenuePerBedCarrots</f>
+        <v/>
+      </c>
+      <c r="I57" s="15">
+        <f>H57-F57</f>
+        <v/>
+      </c>
+      <c r="J57" s="15">
+        <f>A57*RevenuePerBedCarrots-E57-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K57" s="15">
+        <f>(MIN(((TotalLaborHours-LaborHoursCarrots)+B57),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursCarrots)+B57)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursCarrots)+B56),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursCarrots)+B56)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedCarrots</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="13" t="n">
+        <v>24</v>
+      </c>
+      <c r="B58" s="14">
+        <f>A58*LaborHrsPerBedCarrots*SeasonWeeks*(1+DimReturnsCarrots)^A58</f>
+        <v/>
+      </c>
+      <c r="C58" s="15">
+        <f>MIN(B58,OwnLaborHours)*OwnWageRate+MAX(B58-OwnLaborHours,0)*TempWageRate</f>
+        <v/>
+      </c>
+      <c r="D58" s="15">
+        <f>A58*FertilizerPerBedCarrots</f>
+        <v/>
+      </c>
+      <c r="E58" s="15">
+        <f>C58+D58</f>
+        <v/>
+      </c>
+      <c r="F58" s="15">
+        <f>E58-E57</f>
+        <v/>
+      </c>
+      <c r="G58" s="15">
+        <f>E58/A58</f>
+        <v/>
+      </c>
+      <c r="H58" s="15">
+        <f>RevenuePerBedCarrots</f>
+        <v/>
+      </c>
+      <c r="I58" s="15">
+        <f>H58-F58</f>
+        <v/>
+      </c>
+      <c r="J58" s="15">
+        <f>A58*RevenuePerBedCarrots-E58-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K58" s="15">
+        <f>(MIN(((TotalLaborHours-LaborHoursCarrots)+B58),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursCarrots)+B58)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursCarrots)+B57),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursCarrots)+B57)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedCarrots</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="12" t="inlineStr">
         <is>
           <t>Mesclun</t>
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="12" t="inlineStr">
+    <row r="62">
+      <c r="A62" s="12" t="inlineStr">
         <is>
           <t>Beds (q)</t>
         </is>
       </c>
-      <c r="B58" s="12" t="inlineStr">
+      <c r="B62" s="12" t="inlineStr">
         <is>
           <t>Labor hours</t>
         </is>
       </c>
-      <c r="C58" s="12" t="inlineStr">
+      <c r="C62" s="12" t="inlineStr">
         <is>
           <t>Labor cost</t>
         </is>
       </c>
-      <c r="D58" s="12" t="inlineStr">
+      <c r="D62" s="12" t="inlineStr">
         <is>
           <t>Fertilizer cost</t>
         </is>
       </c>
-      <c r="E58" s="12" t="inlineStr">
+      <c r="E62" s="12" t="inlineStr">
         <is>
           <t>Variable cost</t>
         </is>
       </c>
-      <c r="F58" s="12" t="inlineStr">
-        <is>
-          <t>MC</t>
-        </is>
-      </c>
-      <c r="G58" s="12" t="inlineStr">
+      <c r="F62" s="12" t="inlineStr">
+        <is>
+          <t>MC standalone</t>
+        </is>
+      </c>
+      <c r="G62" s="12" t="inlineStr">
         <is>
           <t>AVC</t>
         </is>
       </c>
-      <c r="H58" s="12" t="inlineStr">
+      <c r="H62" s="12" t="inlineStr">
         <is>
           <t>Price</t>
         </is>
       </c>
-      <c r="I58" s="12" t="inlineStr">
+      <c r="I62" s="12" t="inlineStr">
         <is>
           <t>Price − MC</t>
         </is>
       </c>
-      <c r="J58" s="12" t="inlineStr">
+      <c r="J62" s="12" t="inlineStr">
         <is>
           <t>Standalone profit</t>
         </is>
       </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="B59" s="3">
-        <f>A59*LaborHrsPerBedMesclun*SeasonWeeks*(1+DimReturnsMesclun)^A59</f>
-        <v/>
-      </c>
-      <c r="C59" s="4">
-        <f>MIN(B59,OwnLaborHours)*OwnWageRate+MAX(B59-OwnLaborHours,0)*TempWageRate</f>
-        <v/>
-      </c>
-      <c r="D59" s="4">
-        <f>A59*FertilizerPerBedMesclun</f>
-        <v/>
-      </c>
-      <c r="E59" s="4">
-        <f>C59+D59</f>
-        <v/>
-      </c>
-      <c r="H59" s="4">
-        <f>RevenuePerBedMesclun</f>
-        <v/>
-      </c>
-      <c r="J59" s="4">
-        <f>A59*H59-E59-FixedCosts</f>
-        <v/>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B60" s="3">
-        <f>A60*LaborHrsPerBedMesclun*SeasonWeeks*(1+DimReturnsMesclun)^A60</f>
-        <v/>
-      </c>
-      <c r="C60" s="4">
-        <f>MIN(B60,OwnLaborHours)*OwnWageRate+MAX(B60-OwnLaborHours,0)*TempWageRate</f>
-        <v/>
-      </c>
-      <c r="D60" s="4">
-        <f>A60*FertilizerPerBedMesclun</f>
-        <v/>
-      </c>
-      <c r="E60" s="4">
-        <f>C60+D60</f>
-        <v/>
-      </c>
-      <c r="F60" s="4">
-        <f>E60-E59</f>
-        <v/>
-      </c>
-      <c r="G60" s="4">
-        <f>E60/A60</f>
-        <v/>
-      </c>
-      <c r="H60" s="4">
-        <f>RevenuePerBedMesclun</f>
-        <v/>
-      </c>
-      <c r="I60" s="4">
-        <f>H60-F60</f>
-        <v/>
-      </c>
-      <c r="J60" s="4">
-        <f>A60*H60-E60-FixedCosts</f>
-        <v/>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B61" s="3">
-        <f>A61*LaborHrsPerBedMesclun*SeasonWeeks*(1+DimReturnsMesclun)^A61</f>
-        <v/>
-      </c>
-      <c r="C61" s="4">
-        <f>MIN(B61,OwnLaborHours)*OwnWageRate+MAX(B61-OwnLaborHours,0)*TempWageRate</f>
-        <v/>
-      </c>
-      <c r="D61" s="4">
-        <f>A61*FertilizerPerBedMesclun</f>
-        <v/>
-      </c>
-      <c r="E61" s="4">
-        <f>C61+D61</f>
-        <v/>
-      </c>
-      <c r="F61" s="4">
-        <f>E61-E60</f>
-        <v/>
-      </c>
-      <c r="G61" s="4">
-        <f>E61/A61</f>
-        <v/>
-      </c>
-      <c r="H61" s="4">
-        <f>RevenuePerBedMesclun</f>
-        <v/>
-      </c>
-      <c r="I61" s="4">
-        <f>H61-F61</f>
-        <v/>
-      </c>
-      <c r="J61" s="4">
-        <f>A61*H61-E61-FixedCosts</f>
-        <v/>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="B62" s="3">
-        <f>A62*LaborHrsPerBedMesclun*SeasonWeeks*(1+DimReturnsMesclun)^A62</f>
-        <v/>
-      </c>
-      <c r="C62" s="4">
-        <f>MIN(B62,OwnLaborHours)*OwnWageRate+MAX(B62-OwnLaborHours,0)*TempWageRate</f>
-        <v/>
-      </c>
-      <c r="D62" s="4">
-        <f>A62*FertilizerPerBedMesclun</f>
-        <v/>
-      </c>
-      <c r="E62" s="4">
-        <f>C62+D62</f>
-        <v/>
-      </c>
-      <c r="F62" s="4">
-        <f>E62-E61</f>
-        <v/>
-      </c>
-      <c r="G62" s="4">
-        <f>E62/A62</f>
-        <v/>
-      </c>
-      <c r="H62" s="4">
-        <f>RevenuePerBedMesclun</f>
-        <v/>
-      </c>
-      <c r="I62" s="4">
-        <f>H62-F62</f>
-        <v/>
-      </c>
-      <c r="J62" s="4">
-        <f>A62*H62-E62-FixedCosts</f>
-        <v/>
+      <c r="K62" s="12" t="inlineStr">
+        <is>
+          <t>MC in solved mix</t>
+        </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="B63" s="3">
         <f>A63*LaborHrsPerBedMesclun*SeasonWeeks*(1+DimReturnsMesclun)^A63</f>
@@ -4066,30 +4378,14 @@
         <f>C63+D63</f>
         <v/>
       </c>
-      <c r="F63" s="4">
-        <f>E63-E62</f>
-        <v/>
-      </c>
-      <c r="G63" s="4">
-        <f>E63/A63</f>
-        <v/>
-      </c>
-      <c r="H63" s="4">
-        <f>RevenuePerBedMesclun</f>
-        <v/>
-      </c>
-      <c r="I63" s="4">
-        <f>H63-F63</f>
-        <v/>
-      </c>
       <c r="J63" s="4">
-        <f>A63*H63-E63-FixedCosts</f>
+        <f>A63*RevenuePerBedMesclun-E63-FixedCosts</f>
         <v/>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="B64" s="3">
         <f>A64*LaborHrsPerBedMesclun*SeasonWeeks*(1+DimReturnsMesclun)^A64</f>
@@ -4124,13 +4420,17 @@
         <v/>
       </c>
       <c r="J64" s="4">
-        <f>A64*H64-E64-FixedCosts</f>
+        <f>A64*RevenuePerBedMesclun-E64-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K64" s="4">
+        <f>(MIN(((TotalLaborHours-LaborHoursMesclun)+B64),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursMesclun)+B64)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursMesclun)+B63),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursMesclun)+B63)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedMesclun</f>
         <v/>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="B65" s="3">
         <f>A65*LaborHrsPerBedMesclun*SeasonWeeks*(1+DimReturnsMesclun)^A65</f>
@@ -4165,13 +4465,17 @@
         <v/>
       </c>
       <c r="J65" s="4">
-        <f>A65*H65-E65-FixedCosts</f>
+        <f>A65*RevenuePerBedMesclun-E65-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K65" s="4">
+        <f>(MIN(((TotalLaborHours-LaborHoursMesclun)+B65),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursMesclun)+B65)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursMesclun)+B64),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursMesclun)+B64)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedMesclun</f>
         <v/>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="B66" s="3">
         <f>A66*LaborHrsPerBedMesclun*SeasonWeeks*(1+DimReturnsMesclun)^A66</f>
@@ -4206,13 +4510,17 @@
         <v/>
       </c>
       <c r="J66" s="4">
-        <f>A66*H66-E66-FixedCosts</f>
+        <f>A66*RevenuePerBedMesclun-E66-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K66" s="4">
+        <f>(MIN(((TotalLaborHours-LaborHoursMesclun)+B66),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursMesclun)+B66)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursMesclun)+B65),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursMesclun)+B65)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedMesclun</f>
         <v/>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="B67" s="3">
         <f>A67*LaborHrsPerBedMesclun*SeasonWeeks*(1+DimReturnsMesclun)^A67</f>
@@ -4247,13 +4555,17 @@
         <v/>
       </c>
       <c r="J67" s="4">
-        <f>A67*H67-E67-FixedCosts</f>
+        <f>A67*RevenuePerBedMesclun-E67-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K67" s="4">
+        <f>(MIN(((TotalLaborHours-LaborHoursMesclun)+B67),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursMesclun)+B67)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursMesclun)+B66),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursMesclun)+B66)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedMesclun</f>
         <v/>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="B68" s="3">
         <f>A68*LaborHrsPerBedMesclun*SeasonWeeks*(1+DimReturnsMesclun)^A68</f>
@@ -4288,13 +4600,17 @@
         <v/>
       </c>
       <c r="J68" s="4">
-        <f>A68*H68-E68-FixedCosts</f>
+        <f>A68*RevenuePerBedMesclun-E68-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K68" s="4">
+        <f>(MIN(((TotalLaborHours-LaborHoursMesclun)+B68),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursMesclun)+B68)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursMesclun)+B67),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursMesclun)+B67)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedMesclun</f>
         <v/>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="B69" s="3">
         <f>A69*LaborHrsPerBedMesclun*SeasonWeeks*(1+DimReturnsMesclun)^A69</f>
@@ -4329,13 +4645,17 @@
         <v/>
       </c>
       <c r="J69" s="4">
-        <f>A69*H69-E69-FixedCosts</f>
+        <f>A69*RevenuePerBedMesclun-E69-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K69" s="4">
+        <f>(MIN(((TotalLaborHours-LaborHoursMesclun)+B69),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursMesclun)+B69)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursMesclun)+B68),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursMesclun)+B68)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedMesclun</f>
         <v/>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="B70" s="3">
         <f>A70*LaborHrsPerBedMesclun*SeasonWeeks*(1+DimReturnsMesclun)^A70</f>
@@ -4370,13 +4690,17 @@
         <v/>
       </c>
       <c r="J70" s="4">
-        <f>A70*H70-E70-FixedCosts</f>
+        <f>A70*RevenuePerBedMesclun-E70-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K70" s="4">
+        <f>(MIN(((TotalLaborHours-LaborHoursMesclun)+B70),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursMesclun)+B70)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursMesclun)+B69),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursMesclun)+B69)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedMesclun</f>
         <v/>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B71" s="3">
         <f>A71*LaborHrsPerBedMesclun*SeasonWeeks*(1+DimReturnsMesclun)^A71</f>
@@ -4411,13 +4735,17 @@
         <v/>
       </c>
       <c r="J71" s="4">
-        <f>A71*H71-E71-FixedCosts</f>
+        <f>A71*RevenuePerBedMesclun-E71-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K71" s="4">
+        <f>(MIN(((TotalLaborHours-LaborHoursMesclun)+B71),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursMesclun)+B71)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursMesclun)+B70),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursMesclun)+B70)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedMesclun</f>
         <v/>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B72" s="3">
         <f>A72*LaborHrsPerBedMesclun*SeasonWeeks*(1+DimReturnsMesclun)^A72</f>
@@ -4452,13 +4780,17 @@
         <v/>
       </c>
       <c r="J72" s="4">
-        <f>A72*H72-E72-FixedCosts</f>
+        <f>A72*RevenuePerBedMesclun-E72-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K72" s="4">
+        <f>(MIN(((TotalLaborHours-LaborHoursMesclun)+B72),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursMesclun)+B72)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursMesclun)+B71),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursMesclun)+B71)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedMesclun</f>
         <v/>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="B73" s="3">
         <f>A73*LaborHrsPerBedMesclun*SeasonWeeks*(1+DimReturnsMesclun)^A73</f>
@@ -4493,13 +4825,17 @@
         <v/>
       </c>
       <c r="J73" s="4">
-        <f>A73*H73-E73-FixedCosts</f>
+        <f>A73*RevenuePerBedMesclun-E73-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K73" s="4">
+        <f>(MIN(((TotalLaborHours-LaborHoursMesclun)+B73),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursMesclun)+B73)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursMesclun)+B72),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursMesclun)+B72)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedMesclun</f>
         <v/>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B74" s="3">
         <f>A74*LaborHrsPerBedMesclun*SeasonWeeks*(1+DimReturnsMesclun)^A74</f>
@@ -4534,13 +4870,17 @@
         <v/>
       </c>
       <c r="J74" s="4">
-        <f>A74*H74-E74-FixedCosts</f>
+        <f>A74*RevenuePerBedMesclun-E74-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K74" s="4">
+        <f>(MIN(((TotalLaborHours-LaborHoursMesclun)+B74),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursMesclun)+B74)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursMesclun)+B73),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursMesclun)+B73)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedMesclun</f>
         <v/>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="B75" s="3">
         <f>A75*LaborHrsPerBedMesclun*SeasonWeeks*(1+DimReturnsMesclun)^A75</f>
@@ -4575,13 +4915,17 @@
         <v/>
       </c>
       <c r="J75" s="4">
-        <f>A75*H75-E75-FixedCosts</f>
+        <f>A75*RevenuePerBedMesclun-E75-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K75" s="4">
+        <f>(MIN(((TotalLaborHours-LaborHoursMesclun)+B75),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursMesclun)+B75)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursMesclun)+B74),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursMesclun)+B74)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedMesclun</f>
         <v/>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="B76" s="3">
         <f>A76*LaborHrsPerBedMesclun*SeasonWeeks*(1+DimReturnsMesclun)^A76</f>
@@ -4616,13 +4960,17 @@
         <v/>
       </c>
       <c r="J76" s="4">
-        <f>A76*H76-E76-FixedCosts</f>
+        <f>A76*RevenuePerBedMesclun-E76-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K76" s="4">
+        <f>(MIN(((TotalLaborHours-LaborHoursMesclun)+B76),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursMesclun)+B76)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursMesclun)+B75),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursMesclun)+B75)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedMesclun</f>
         <v/>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="B77" s="3">
         <f>A77*LaborHrsPerBedMesclun*SeasonWeeks*(1+DimReturnsMesclun)^A77</f>
@@ -4657,13 +5005,17 @@
         <v/>
       </c>
       <c r="J77" s="4">
-        <f>A77*H77-E77-FixedCosts</f>
+        <f>A77*RevenuePerBedMesclun-E77-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K77" s="4">
+        <f>(MIN(((TotalLaborHours-LaborHoursMesclun)+B77),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursMesclun)+B77)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursMesclun)+B76),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursMesclun)+B76)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedMesclun</f>
         <v/>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="B78" s="3">
         <f>A78*LaborHrsPerBedMesclun*SeasonWeeks*(1+DimReturnsMesclun)^A78</f>
@@ -4698,13 +5050,17 @@
         <v/>
       </c>
       <c r="J78" s="4">
-        <f>A78*H78-E78-FixedCosts</f>
+        <f>A78*RevenuePerBedMesclun-E78-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K78" s="4">
+        <f>(MIN(((TotalLaborHours-LaborHoursMesclun)+B78),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursMesclun)+B78)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursMesclun)+B77),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursMesclun)+B77)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedMesclun</f>
         <v/>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="B79" s="3">
         <f>A79*LaborHrsPerBedMesclun*SeasonWeeks*(1+DimReturnsMesclun)^A79</f>
@@ -4739,13 +5095,17 @@
         <v/>
       </c>
       <c r="J79" s="4">
-        <f>A79*H79-E79-FixedCosts</f>
+        <f>A79*RevenuePerBedMesclun-E79-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K79" s="4">
+        <f>(MIN(((TotalLaborHours-LaborHoursMesclun)+B79),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursMesclun)+B79)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursMesclun)+B78),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursMesclun)+B78)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedMesclun</f>
         <v/>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B80" s="3">
         <f>A80*LaborHrsPerBedMesclun*SeasonWeeks*(1+DimReturnsMesclun)^A80</f>
@@ -4780,13 +5140,17 @@
         <v/>
       </c>
       <c r="J80" s="4">
-        <f>A80*H80-E80-FixedCosts</f>
+        <f>A80*RevenuePerBedMesclun-E80-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K80" s="4">
+        <f>(MIN(((TotalLaborHours-LaborHoursMesclun)+B80),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursMesclun)+B80)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursMesclun)+B79),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursMesclun)+B79)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedMesclun</f>
         <v/>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="B81" s="3">
         <f>A81*LaborHrsPerBedMesclun*SeasonWeeks*(1+DimReturnsMesclun)^A81</f>
@@ -4821,13 +5185,17 @@
         <v/>
       </c>
       <c r="J81" s="4">
-        <f>A81*H81-E81-FixedCosts</f>
+        <f>A81*RevenuePerBedMesclun-E81-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K81" s="4">
+        <f>(MIN(((TotalLaborHours-LaborHoursMesclun)+B81),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursMesclun)+B81)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursMesclun)+B80),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursMesclun)+B80)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedMesclun</f>
         <v/>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="B82" s="3">
         <f>A82*LaborHrsPerBedMesclun*SeasonWeeks*(1+DimReturnsMesclun)^A82</f>
@@ -4862,13 +5230,17 @@
         <v/>
       </c>
       <c r="J82" s="4">
-        <f>A82*H82-E82-FixedCosts</f>
+        <f>A82*RevenuePerBedMesclun-E82-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K82" s="4">
+        <f>(MIN(((TotalLaborHours-LaborHoursMesclun)+B82),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursMesclun)+B82)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursMesclun)+B81),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursMesclun)+B81)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedMesclun</f>
         <v/>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="B83" s="3">
         <f>A83*LaborHrsPerBedMesclun*SeasonWeeks*(1+DimReturnsMesclun)^A83</f>
@@ -4903,13 +5275,17 @@
         <v/>
       </c>
       <c r="J83" s="4">
-        <f>A83*H83-E83-FixedCosts</f>
+        <f>A83*RevenuePerBedMesclun-E83-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K83" s="4">
+        <f>(MIN(((TotalLaborHours-LaborHoursMesclun)+B83),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursMesclun)+B83)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursMesclun)+B82),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursMesclun)+B82)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedMesclun</f>
         <v/>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B84" s="3">
         <f>A84*LaborHrsPerBedMesclun*SeasonWeeks*(1+DimReturnsMesclun)^A84</f>
@@ -4944,13 +5320,17 @@
         <v/>
       </c>
       <c r="J84" s="4">
-        <f>A84*H84-E84-FixedCosts</f>
+        <f>A84*RevenuePerBedMesclun-E84-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K84" s="4">
+        <f>(MIN(((TotalLaborHours-LaborHoursMesclun)+B84),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursMesclun)+B84)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursMesclun)+B83),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursMesclun)+B83)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedMesclun</f>
         <v/>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B85" s="3">
         <f>A85*LaborHrsPerBedMesclun*SeasonWeeks*(1+DimReturnsMesclun)^A85</f>
@@ -4985,13 +5365,17 @@
         <v/>
       </c>
       <c r="J85" s="4">
-        <f>A85*H85-E85-FixedCosts</f>
+        <f>A85*RevenuePerBedMesclun-E85-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K85" s="4">
+        <f>(MIN(((TotalLaborHours-LaborHoursMesclun)+B85),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursMesclun)+B85)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursMesclun)+B84),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursMesclun)+B84)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedMesclun</f>
         <v/>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="n">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="B86" s="3">
         <f>A86*LaborHrsPerBedMesclun*SeasonWeeks*(1+DimReturnsMesclun)^A86</f>
@@ -5026,13 +5410,17 @@
         <v/>
       </c>
       <c r="J86" s="4">
-        <f>A86*H86-E86-FixedCosts</f>
+        <f>A86*RevenuePerBedMesclun-E86-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K86" s="4">
+        <f>(MIN(((TotalLaborHours-LaborHoursMesclun)+B86),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursMesclun)+B86)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursMesclun)+B85),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursMesclun)+B85)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedMesclun</f>
         <v/>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="n">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="B87" s="3">
         <f>A87*LaborHrsPerBedMesclun*SeasonWeeks*(1+DimReturnsMesclun)^A87</f>
@@ -5067,13 +5455,17 @@
         <v/>
       </c>
       <c r="J87" s="4">
-        <f>A87*H87-E87-FixedCosts</f>
+        <f>A87*RevenuePerBedMesclun-E87-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K87" s="4">
+        <f>(MIN(((TotalLaborHours-LaborHoursMesclun)+B87),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursMesclun)+B87)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursMesclun)+B86),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursMesclun)+B86)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedMesclun</f>
         <v/>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="n">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B88" s="3">
         <f>A88*LaborHrsPerBedMesclun*SeasonWeeks*(1+DimReturnsMesclun)^A88</f>
@@ -5108,13 +5500,17 @@
         <v/>
       </c>
       <c r="J88" s="4">
-        <f>A88*H88-E88-FixedCosts</f>
+        <f>A88*RevenuePerBedMesclun-E88-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K88" s="4">
+        <f>(MIN(((TotalLaborHours-LaborHoursMesclun)+B88),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursMesclun)+B88)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursMesclun)+B87),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursMesclun)+B87)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedMesclun</f>
         <v/>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="n">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="B89" s="3">
         <f>A89*LaborHrsPerBedMesclun*SeasonWeeks*(1+DimReturnsMesclun)^A89</f>
@@ -5149,7 +5545,371 @@
         <v/>
       </c>
       <c r="J89" s="4">
-        <f>A89*H89-E89-FixedCosts</f>
+        <f>A89*RevenuePerBedMesclun-E89-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K89" s="4">
+        <f>(MIN(((TotalLaborHours-LaborHoursMesclun)+B89),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursMesclun)+B89)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursMesclun)+B88),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursMesclun)+B88)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedMesclun</f>
+        <v/>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="B90" s="3">
+        <f>A90*LaborHrsPerBedMesclun*SeasonWeeks*(1+DimReturnsMesclun)^A90</f>
+        <v/>
+      </c>
+      <c r="C90" s="4">
+        <f>MIN(B90,OwnLaborHours)*OwnWageRate+MAX(B90-OwnLaborHours,0)*TempWageRate</f>
+        <v/>
+      </c>
+      <c r="D90" s="4">
+        <f>A90*FertilizerPerBedMesclun</f>
+        <v/>
+      </c>
+      <c r="E90" s="4">
+        <f>C90+D90</f>
+        <v/>
+      </c>
+      <c r="F90" s="4">
+        <f>E90-E89</f>
+        <v/>
+      </c>
+      <c r="G90" s="4">
+        <f>E90/A90</f>
+        <v/>
+      </c>
+      <c r="H90" s="4">
+        <f>RevenuePerBedMesclun</f>
+        <v/>
+      </c>
+      <c r="I90" s="4">
+        <f>H90-F90</f>
+        <v/>
+      </c>
+      <c r="J90" s="4">
+        <f>A90*RevenuePerBedMesclun-E90-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K90" s="4">
+        <f>(MIN(((TotalLaborHours-LaborHoursMesclun)+B90),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursMesclun)+B90)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursMesclun)+B89),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursMesclun)+B89)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedMesclun</f>
+        <v/>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="B91" s="3">
+        <f>A91*LaborHrsPerBedMesclun*SeasonWeeks*(1+DimReturnsMesclun)^A91</f>
+        <v/>
+      </c>
+      <c r="C91" s="4">
+        <f>MIN(B91,OwnLaborHours)*OwnWageRate+MAX(B91-OwnLaborHours,0)*TempWageRate</f>
+        <v/>
+      </c>
+      <c r="D91" s="4">
+        <f>A91*FertilizerPerBedMesclun</f>
+        <v/>
+      </c>
+      <c r="E91" s="4">
+        <f>C91+D91</f>
+        <v/>
+      </c>
+      <c r="F91" s="4">
+        <f>E91-E90</f>
+        <v/>
+      </c>
+      <c r="G91" s="4">
+        <f>E91/A91</f>
+        <v/>
+      </c>
+      <c r="H91" s="4">
+        <f>RevenuePerBedMesclun</f>
+        <v/>
+      </c>
+      <c r="I91" s="4">
+        <f>H91-F91</f>
+        <v/>
+      </c>
+      <c r="J91" s="4">
+        <f>A91*RevenuePerBedMesclun-E91-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K91" s="4">
+        <f>(MIN(((TotalLaborHours-LaborHoursMesclun)+B91),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursMesclun)+B91)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursMesclun)+B90),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursMesclun)+B90)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedMesclun</f>
+        <v/>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="B92" s="3">
+        <f>A92*LaborHrsPerBedMesclun*SeasonWeeks*(1+DimReturnsMesclun)^A92</f>
+        <v/>
+      </c>
+      <c r="C92" s="4">
+        <f>MIN(B92,OwnLaborHours)*OwnWageRate+MAX(B92-OwnLaborHours,0)*TempWageRate</f>
+        <v/>
+      </c>
+      <c r="D92" s="4">
+        <f>A92*FertilizerPerBedMesclun</f>
+        <v/>
+      </c>
+      <c r="E92" s="4">
+        <f>C92+D92</f>
+        <v/>
+      </c>
+      <c r="F92" s="4">
+        <f>E92-E91</f>
+        <v/>
+      </c>
+      <c r="G92" s="4">
+        <f>E92/A92</f>
+        <v/>
+      </c>
+      <c r="H92" s="4">
+        <f>RevenuePerBedMesclun</f>
+        <v/>
+      </c>
+      <c r="I92" s="4">
+        <f>H92-F92</f>
+        <v/>
+      </c>
+      <c r="J92" s="4">
+        <f>A92*RevenuePerBedMesclun-E92-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K92" s="4">
+        <f>(MIN(((TotalLaborHours-LaborHoursMesclun)+B92),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursMesclun)+B92)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursMesclun)+B91),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursMesclun)+B91)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedMesclun</f>
+        <v/>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="B93" s="3">
+        <f>A93*LaborHrsPerBedMesclun*SeasonWeeks*(1+DimReturnsMesclun)^A93</f>
+        <v/>
+      </c>
+      <c r="C93" s="4">
+        <f>MIN(B93,OwnLaborHours)*OwnWageRate+MAX(B93-OwnLaborHours,0)*TempWageRate</f>
+        <v/>
+      </c>
+      <c r="D93" s="4">
+        <f>A93*FertilizerPerBedMesclun</f>
+        <v/>
+      </c>
+      <c r="E93" s="4">
+        <f>C93+D93</f>
+        <v/>
+      </c>
+      <c r="F93" s="4">
+        <f>E93-E92</f>
+        <v/>
+      </c>
+      <c r="G93" s="4">
+        <f>E93/A93</f>
+        <v/>
+      </c>
+      <c r="H93" s="4">
+        <f>RevenuePerBedMesclun</f>
+        <v/>
+      </c>
+      <c r="I93" s="4">
+        <f>H93-F93</f>
+        <v/>
+      </c>
+      <c r="J93" s="4">
+        <f>A93*RevenuePerBedMesclun-E93-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K93" s="4">
+        <f>(MIN(((TotalLaborHours-LaborHoursMesclun)+B93),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursMesclun)+B93)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursMesclun)+B92),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursMesclun)+B92)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedMesclun</f>
+        <v/>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="13" t="n">
+        <v>31</v>
+      </c>
+      <c r="B94" s="14">
+        <f>A94*LaborHrsPerBedMesclun*SeasonWeeks*(1+DimReturnsMesclun)^A94</f>
+        <v/>
+      </c>
+      <c r="C94" s="15">
+        <f>MIN(B94,OwnLaborHours)*OwnWageRate+MAX(B94-OwnLaborHours,0)*TempWageRate</f>
+        <v/>
+      </c>
+      <c r="D94" s="15">
+        <f>A94*FertilizerPerBedMesclun</f>
+        <v/>
+      </c>
+      <c r="E94" s="15">
+        <f>C94+D94</f>
+        <v/>
+      </c>
+      <c r="F94" s="15">
+        <f>E94-E93</f>
+        <v/>
+      </c>
+      <c r="G94" s="15">
+        <f>E94/A94</f>
+        <v/>
+      </c>
+      <c r="H94" s="15">
+        <f>RevenuePerBedMesclun</f>
+        <v/>
+      </c>
+      <c r="I94" s="15">
+        <f>H94-F94</f>
+        <v/>
+      </c>
+      <c r="J94" s="15">
+        <f>A94*RevenuePerBedMesclun-E94-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K94" s="15">
+        <f>(MIN(((TotalLaborHours-LaborHoursMesclun)+B94),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursMesclun)+B94)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursMesclun)+B93),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursMesclun)+B93)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedMesclun</f>
+        <v/>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="13" t="n">
+        <v>32</v>
+      </c>
+      <c r="B95" s="14">
+        <f>A95*LaborHrsPerBedMesclun*SeasonWeeks*(1+DimReturnsMesclun)^A95</f>
+        <v/>
+      </c>
+      <c r="C95" s="15">
+        <f>MIN(B95,OwnLaborHours)*OwnWageRate+MAX(B95-OwnLaborHours,0)*TempWageRate</f>
+        <v/>
+      </c>
+      <c r="D95" s="15">
+        <f>A95*FertilizerPerBedMesclun</f>
+        <v/>
+      </c>
+      <c r="E95" s="15">
+        <f>C95+D95</f>
+        <v/>
+      </c>
+      <c r="F95" s="15">
+        <f>E95-E94</f>
+        <v/>
+      </c>
+      <c r="G95" s="15">
+        <f>E95/A95</f>
+        <v/>
+      </c>
+      <c r="H95" s="15">
+        <f>RevenuePerBedMesclun</f>
+        <v/>
+      </c>
+      <c r="I95" s="15">
+        <f>H95-F95</f>
+        <v/>
+      </c>
+      <c r="J95" s="15">
+        <f>A95*RevenuePerBedMesclun-E95-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K95" s="15">
+        <f>(MIN(((TotalLaborHours-LaborHoursMesclun)+B95),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursMesclun)+B95)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursMesclun)+B94),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursMesclun)+B94)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedMesclun</f>
+        <v/>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="13" t="n">
+        <v>33</v>
+      </c>
+      <c r="B96" s="14">
+        <f>A96*LaborHrsPerBedMesclun*SeasonWeeks*(1+DimReturnsMesclun)^A96</f>
+        <v/>
+      </c>
+      <c r="C96" s="15">
+        <f>MIN(B96,OwnLaborHours)*OwnWageRate+MAX(B96-OwnLaborHours,0)*TempWageRate</f>
+        <v/>
+      </c>
+      <c r="D96" s="15">
+        <f>A96*FertilizerPerBedMesclun</f>
+        <v/>
+      </c>
+      <c r="E96" s="15">
+        <f>C96+D96</f>
+        <v/>
+      </c>
+      <c r="F96" s="15">
+        <f>E96-E95</f>
+        <v/>
+      </c>
+      <c r="G96" s="15">
+        <f>E96/A96</f>
+        <v/>
+      </c>
+      <c r="H96" s="15">
+        <f>RevenuePerBedMesclun</f>
+        <v/>
+      </c>
+      <c r="I96" s="15">
+        <f>H96-F96</f>
+        <v/>
+      </c>
+      <c r="J96" s="15">
+        <f>A96*RevenuePerBedMesclun-E96-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K96" s="15">
+        <f>(MIN(((TotalLaborHours-LaborHoursMesclun)+B96),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursMesclun)+B96)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursMesclun)+B95),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursMesclun)+B95)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedMesclun</f>
+        <v/>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="13" t="n">
+        <v>34</v>
+      </c>
+      <c r="B97" s="14">
+        <f>A97*LaborHrsPerBedMesclun*SeasonWeeks*(1+DimReturnsMesclun)^A97</f>
+        <v/>
+      </c>
+      <c r="C97" s="15">
+        <f>MIN(B97,OwnLaborHours)*OwnWageRate+MAX(B97-OwnLaborHours,0)*TempWageRate</f>
+        <v/>
+      </c>
+      <c r="D97" s="15">
+        <f>A97*FertilizerPerBedMesclun</f>
+        <v/>
+      </c>
+      <c r="E97" s="15">
+        <f>C97+D97</f>
+        <v/>
+      </c>
+      <c r="F97" s="15">
+        <f>E97-E96</f>
+        <v/>
+      </c>
+      <c r="G97" s="15">
+        <f>E97/A97</f>
+        <v/>
+      </c>
+      <c r="H97" s="15">
+        <f>RevenuePerBedMesclun</f>
+        <v/>
+      </c>
+      <c r="I97" s="15">
+        <f>H97-F97</f>
+        <v/>
+      </c>
+      <c r="J97" s="15">
+        <f>A97*RevenuePerBedMesclun-E97-FixedCosts</f>
+        <v/>
+      </c>
+      <c r="K97" s="15">
+        <f>(MIN(((TotalLaborHours-LaborHoursMesclun)+B97),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursMesclun)+B97)-OwnLaborHours,0)*TempWageRate)-(MIN(((TotalLaborHours-LaborHoursMesclun)+B96),OwnLaborHours)*OwnWageRate+MAX(((TotalLaborHours-LaborHoursMesclun)+B96)-OwnLaborHours,0)*TempWageRate)+FertilizerPerBedMesclun</f>
         <v/>
       </c>
     </row>

</xml_diff>